<commit_message>
Altera cores - mediaMaisAltaeMaisBaixa
.
</commit_message>
<xml_diff>
--- a/Avaliacao.xlsx
+++ b/Avaliacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisf\OneDrive\Documentos\ESA 2021-22\Formacao GitHub\Projeto\GrelhaExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B2DDDA-F9CD-44BB-9F61-AD156768B19C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A467E9-C34D-4611-BB58-038AB9CF7EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4416" yWindow="0" windowWidth="12024" windowHeight="12240" xr2:uid="{9C8FBE48-8480-45E8-A2FE-8EF4A5DD2B63}"/>
   </bookViews>
@@ -81,7 +81,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -112,6 +112,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="21">
     <border>
@@ -437,10 +443,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -465,6 +467,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -805,21 +811,21 @@
     <row r="5" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C6" s="10"/>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="G6" s="20" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="16" t="s">
         <v>0</v>
       </c>
       <c r="D7" s="7">
@@ -831,13 +837,13 @@
       <c r="F7" s="9">
         <v>14</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="19">
         <f>AVERAGE(D7:F7)</f>
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="17" t="s">
         <v>1</v>
       </c>
       <c r="D8" s="2">
@@ -849,13 +855,13 @@
       <c r="F8" s="3">
         <v>6</v>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="19">
         <f t="shared" ref="G8:G10" si="0">AVERAGE(D8:F8)</f>
         <v>9.3333333333333339</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="17" t="s">
         <v>2</v>
       </c>
       <c r="D9" s="2">
@@ -867,13 +873,13 @@
       <c r="F9" s="3">
         <v>12</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="19">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="18" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="6">
@@ -885,27 +891,27 @@
       <c r="F10" s="5">
         <v>14</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="19">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="14"/>
+      <c r="C12" s="22"/>
       <c r="D12" s="12">
         <f>MAX(G7:G10)</f>
         <v>14</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="16"/>
+      <c r="C13" s="24"/>
       <c r="D13" s="11">
         <f>MIN(G7:G10)</f>
         <v>9.3333333333333339</v>

</xml_diff>